<commit_message>
Emoji File, Wk 3 Orders, and Fixes
Create an Emoji excel file to help with seeing what emojis will look like in Excel.
Downloaded Wk 3 csv and pdf order files.
Updated process to run on 4/6/2022 file with default orders. Made a change in default logic to be simpler and only need a single name for 5 FS groups. Identified and fixed issue where customers can select multiple pickup times.
</commit_message>
<xml_diff>
--- a/test_notebooks_R/TestFile.xlsx
+++ b/test_notebooks_R/TestFile.xlsx
@@ -101,7 +101,7 @@
     <t xml:space="preserve">1x1 Loaf Seedy Wheaty Bread</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]1x64 Oz. Milk - Whole</t>
+    <t xml:space="preserve">🐄[*]1x64 Oz. Milk - Whole</t>
   </si>
   <si>
     <t xml:space="preserve">1x1 Pack Boerewors Sausage</t>
@@ -410,7 +410,7 @@
     <t xml:space="preserve">Han, Martha</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]1x64 Ounce 2% MILK</t>
+    <t xml:space="preserve">🐄[*]1x64 Ounce 2% MILK</t>
   </si>
   <si>
     <t xml:space="preserve">1x1 Green Curry Sauce</t>
@@ -500,7 +500,7 @@
     <t xml:space="preserve">Stankovic, Dusica</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]1x64 Ounce Whole MILK</t>
+    <t xml:space="preserve">🐄[*]1x64 Ounce Whole MILK</t>
   </si>
   <si>
     <t xml:space="preserve">🍕[**]1x1 Each Pizza - Tomato Basil Garlic</t>
@@ -539,10 +539,10 @@
     <t xml:space="preserve">1x1 Pint Apple Butter - No Sugar</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]1x64 Oz. Milk - 2%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🥛[*]1x64 Oz. Milk - Creamline</t>
+    <t xml:space="preserve">🐄[*]1x64 Oz. Milk - 2%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">🐄[*]1x64 Oz. Milk - Creamline</t>
   </si>
   <si>
     <t xml:space="preserve">1x2 Lb. Grits</t>
@@ -632,7 +632,7 @@
     <t xml:space="preserve">Waters, Aileen</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]1x64 Ounce 2% MILK-o</t>
+    <t xml:space="preserve">🐄[*]1x64 Ounce 2% MILK-o</t>
   </si>
   <si>
     <t xml:space="preserve">1x1 Pack Gouda - 5 Alarm</t>
@@ -677,7 +677,7 @@
     <t xml:space="preserve">Yau, Caroline &amp; Tim</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]2x64 Ounce Whole MILK-o</t>
+    <t xml:space="preserve">🐄[*]2x64 Ounce Whole MILK-o</t>
   </si>
   <si>
     <t xml:space="preserve">Cooper, Ben</t>
@@ -815,7 +815,7 @@
     <t xml:space="preserve">Levin, Petra</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]6x64 Ounce Whole MILK-o</t>
+    <t xml:space="preserve">🐄[*]6x64 Ounce Whole MILK-o</t>
   </si>
   <si>
     <t xml:space="preserve">Parks, Mary Beth</t>
@@ -950,7 +950,7 @@
     <t xml:space="preserve">Robertson, Janice</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]1x64 Ounce Chocolate MILK</t>
+    <t xml:space="preserve">🐄[*]1x64 Ounce Chocolate MILK</t>
   </si>
   <si>
     <t xml:space="preserve">1x1 Lb. Gnocchi - Potato</t>
@@ -983,7 +983,7 @@
     <t xml:space="preserve">Schaefer, Anneliese</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]2x64 Ounce 2% MILK</t>
+    <t xml:space="preserve">🐄[*]2x64 Ounce 2% MILK</t>
   </si>
   <si>
     <t xml:space="preserve">1x1 Bag Gift - Dine &amp; Dash</t>
@@ -1055,7 +1055,7 @@
     <t xml:space="preserve">Coolman, Audrey</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]1x64 Ounce Skim MILK</t>
+    <t xml:space="preserve">🐄[*]1x64 Ounce Skim MILK</t>
   </si>
   <si>
     <t xml:space="preserve">1x1 Bag Basmati or Jasmine Rice Choice</t>
@@ -1076,7 +1076,7 @@
     <t xml:space="preserve">Piepgrass, Erin</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]2x64 Ounce Creamline MILK</t>
+    <t xml:space="preserve">🐄[*]2x64 Ounce Creamline MILK</t>
   </si>
   <si>
     <t xml:space="preserve">1x64 Ounce CREAM</t>
@@ -1124,7 +1124,7 @@
     <t xml:space="preserve">1 Mini</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]2x64 Ounce Whole MILK</t>
+    <t xml:space="preserve">🐄[*]2x64 Ounce Whole MILK</t>
   </si>
   <si>
     <t xml:space="preserve">1x1 Each Bada Bing - Sub - Frozen</t>
@@ -1421,7 +1421,7 @@
     <t xml:space="preserve">🕒1x2 @5-5:30 UCA UCB UCM UCG Pickup Time</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]2x64 Oz. Milk - 2%</t>
+    <t xml:space="preserve">🐄[*]2x64 Oz. Milk - 2%</t>
   </si>
   <si>
     <t xml:space="preserve">1x1 Bag Bagels - Everything - Frozen</t>
@@ -1493,7 +1493,7 @@
     <t xml:space="preserve">🕒1x3 @5:30-6 UCA UCB UCM UCG Pickup Time</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]1x64 Oz. Milk - Skim</t>
+    <t xml:space="preserve">🐄[*]1x64 Oz. Milk - Skim</t>
   </si>
   <si>
     <t xml:space="preserve">Frank, Debbie</t>
@@ -1583,7 +1583,7 @@
     <t xml:space="preserve">Volkan, Susan</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]1x64 Ounce Skim MILK-o</t>
+    <t xml:space="preserve">🐄[*]1x64 Ounce Skim MILK-o</t>
   </si>
   <si>
     <t xml:space="preserve">1x1 Pack Granola - Vanilla Apricot</t>
@@ -1766,7 +1766,7 @@
     <t xml:space="preserve">1xea. YoBul plain yogurt</t>
   </si>
   <si>
-    <t xml:space="preserve">🥛[*]1x64 Oz. Milk - Chocolate</t>
+    <t xml:space="preserve">🐄[*]1x64 Oz. Milk - Chocolate</t>
   </si>
   <si>
     <t xml:space="preserve">Morley, Deborah</t>

</xml_diff>